<commit_message>
Add 5 new complexes and fix UI bugs
- Add 동천역: 현대홈타운1차, 현대홈타운2차, 동천디이스트, 써니벨리
- Add 성복역: 강남빌리지
- Group filter tabs by station (수지구청/동천/성복)
- Fix 저층제외: filter individual floor entries, not entire group
- Fix "도보 undefined분" → show station name
- Title: 수지구청역 관심 아파트 → 수지 관심 아파트
- Total: 13 complexes, 255 listings

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/listings.xlsx
+++ b/listings.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H172"/>
+  <dimension ref="A1:H256"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -674,7 +674,7 @@
         <v>용인수지신정마을9단지</v>
       </c>
       <c r="B11" t="str">
-        <v>10억 6,000</v>
+        <v>10억 5,000</v>
       </c>
       <c r="C11">
         <v>72</v>
@@ -683,13 +683,13 @@
         <v>901동</v>
       </c>
       <c r="E11" t="str">
-        <v>10/18</v>
+        <v>18/18</v>
       </c>
       <c r="F11" t="str">
         <v>남동향</v>
       </c>
       <c r="G11" t="str">
-        <v>샷시포함올수리 거실확장 중문 수지구청역역세권</v>
+        <v>샷시포함올수리,트인전망,공원,탄천연결,초역세권,입주협의</v>
       </c>
       <c r="H11" t="str">
         <v>naver</v>
@@ -700,22 +700,22 @@
         <v>용인수지신정마을9단지</v>
       </c>
       <c r="B12" t="str">
-        <v>10억 3,000</v>
+        <v>11억 7,000</v>
       </c>
       <c r="C12">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="D12" t="str">
-        <v>905동</v>
+        <v>902동</v>
       </c>
       <c r="E12" t="str">
-        <v>8/18</v>
+        <v>7/20</v>
       </c>
       <c r="F12" t="str">
-        <v>남동향</v>
+        <v>남서향</v>
       </c>
       <c r="G12" t="str">
-        <v>올수리,탄천전망,주차여유,초역세권,공원,4월초부터입주협의</v>
+        <v>정상입주,샷시교체,올수리,방1확장,트인전망,초역세권,학군</v>
       </c>
       <c r="H12" t="str">
         <v>naver</v>
@@ -752,7 +752,7 @@
         <v>용인수지신정마을9단지</v>
       </c>
       <c r="B14" t="str">
-        <v>10억 5,000</v>
+        <v>10억 6,000</v>
       </c>
       <c r="C14">
         <v>72</v>
@@ -761,13 +761,13 @@
         <v>901동</v>
       </c>
       <c r="E14" t="str">
-        <v>18/18</v>
+        <v>10/18</v>
       </c>
       <c r="F14" t="str">
         <v>남동향</v>
       </c>
       <c r="G14" t="str">
-        <v>샷시포함올수리,트인전망,공원,탄천연결,초역세권,입주협의</v>
+        <v>샷시포함올수리 거실확장 중문 수지구청역역세권</v>
       </c>
       <c r="H14" t="str">
         <v>naver</v>
@@ -804,22 +804,22 @@
         <v>용인수지신정마을9단지</v>
       </c>
       <c r="B16" t="str">
-        <v>11억 7,000</v>
+        <v>10억 3,000</v>
       </c>
       <c r="C16">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="D16" t="str">
-        <v>902동</v>
+        <v>905동</v>
       </c>
       <c r="E16" t="str">
-        <v>7/20</v>
+        <v>8/18</v>
       </c>
       <c r="F16" t="str">
-        <v>남서향</v>
+        <v>남동향</v>
       </c>
       <c r="G16" t="str">
-        <v>정상입주,샷시교체,올수리,방1확장,트인전망,초역세권,학군</v>
+        <v>올수리,탄천전망,주차여유,초역세권,공원,4월초부터입주협의</v>
       </c>
       <c r="H16" t="str">
         <v>naver</v>
@@ -856,22 +856,22 @@
         <v>용인수지신정마을9단지</v>
       </c>
       <c r="B18" t="str">
-        <v>10억 3,000</v>
+        <v>10억 4,000</v>
       </c>
       <c r="C18">
         <v>72</v>
       </c>
       <c r="D18" t="str">
-        <v>905동</v>
+        <v>908동</v>
       </c>
       <c r="E18" t="str">
-        <v>16/18</v>
+        <v>13/18</v>
       </c>
       <c r="F18" t="str">
         <v>남동향</v>
       </c>
       <c r="G18" t="str">
-        <v>정상,전체올수리,샷시,수지구청역세권,탄천전망,지하주차장 굿</v>
+        <v>정상입주,로얄동,올수리,깨끗</v>
       </c>
       <c r="H18" t="str">
         <v>naver</v>
@@ -882,22 +882,22 @@
         <v>용인수지신정마을9단지</v>
       </c>
       <c r="B19" t="str">
-        <v>10억 4,000</v>
+        <v>10억 3,000</v>
       </c>
       <c r="C19">
         <v>72</v>
       </c>
       <c r="D19" t="str">
-        <v>908동</v>
+        <v>905동</v>
       </c>
       <c r="E19" t="str">
-        <v>13/18</v>
+        <v>16/18</v>
       </c>
       <c r="F19" t="str">
         <v>남동향</v>
       </c>
       <c r="G19" t="str">
-        <v>정상입주,로얄동,올수리,깨끗</v>
+        <v>정상,전체올수리,샷시,수지구청역세권,탄천전망,지하주차장 굿</v>
       </c>
       <c r="H19" t="str">
         <v>naver</v>
@@ -1194,22 +1194,22 @@
         <v>신정7단지(상록)공무원</v>
       </c>
       <c r="B31" t="str">
-        <v>10억 4,000</v>
+        <v>13억 9,000</v>
       </c>
       <c r="C31">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="D31" t="str">
-        <v>705동</v>
+        <v>704동</v>
       </c>
       <c r="E31" t="str">
-        <v>2/20</v>
+        <v>19/20</v>
       </c>
       <c r="F31" t="str">
         <v>남동향</v>
       </c>
       <c r="G31" t="str">
-        <v>입주일협의가. 중도금이후인테리어가능.2년전 전체적으로 올수리</v>
+        <v>세안고27년9월말, 외부샷시교체,방1확장,내부일부수리,로얄동로얄층</v>
       </c>
       <c r="H31" t="str">
         <v>naver</v>
@@ -1220,22 +1220,22 @@
         <v>신정7단지(상록)공무원</v>
       </c>
       <c r="B32" t="str">
-        <v>13억 9,000</v>
+        <v>14억</v>
       </c>
       <c r="C32">
         <v>109</v>
       </c>
       <c r="D32" t="str">
-        <v>704동</v>
+        <v>701동</v>
       </c>
       <c r="E32" t="str">
-        <v>19/20</v>
+        <v>16/20</v>
       </c>
       <c r="F32" t="str">
         <v>남동향</v>
       </c>
       <c r="G32" t="str">
-        <v>세안고27년9월말, 외부샷시교체,방1확장,내부일부수리,로얄동로얄층</v>
+        <v>예전 올수리 방1 주방확장 초품아 학군최고 신분당선역세권</v>
       </c>
       <c r="H32" t="str">
         <v>naver</v>
@@ -1246,22 +1246,22 @@
         <v>신정7단지(상록)공무원</v>
       </c>
       <c r="B33" t="str">
-        <v>14억</v>
+        <v>10억 4,000</v>
       </c>
       <c r="C33">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="D33" t="str">
-        <v>701동</v>
+        <v>705동</v>
       </c>
       <c r="E33" t="str">
-        <v>16/20</v>
+        <v>2/20</v>
       </c>
       <c r="F33" t="str">
         <v>남동향</v>
       </c>
       <c r="G33" t="str">
-        <v>예전 올수리 방1 주방확장 초품아 학군최고 신분당선역세권</v>
+        <v>주인직접의뢰.로얄동,즉시입주가능.초급매</v>
       </c>
       <c r="H33" t="str">
         <v>naver</v>
@@ -1662,7 +1662,7 @@
         <v>한국</v>
       </c>
       <c r="B49" t="str">
-        <v>12억</v>
+        <v>11억 5,000</v>
       </c>
       <c r="C49">
         <v>105</v>
@@ -1671,13 +1671,13 @@
         <v>103동</v>
       </c>
       <c r="E49" t="str">
-        <v>고/16</v>
+        <v>저/16</v>
       </c>
       <c r="F49" t="str">
         <v>남동향</v>
       </c>
       <c r="G49" t="str">
-        <v>입주가,  샷시포함 올수리되고 깨끗함</v>
+        <v>로얄동 리모델링 추진단지 수지구청역초역세권 입주협의</v>
       </c>
       <c r="H49" t="str">
         <v>naver</v>
@@ -1688,7 +1688,7 @@
         <v>한국</v>
       </c>
       <c r="B50" t="str">
-        <v>11억 5,000</v>
+        <v>12억</v>
       </c>
       <c r="C50">
         <v>105</v>
@@ -1697,13 +1697,13 @@
         <v>103동</v>
       </c>
       <c r="E50" t="str">
-        <v>저/16</v>
+        <v>고/16</v>
       </c>
       <c r="F50" t="str">
         <v>남동향</v>
       </c>
       <c r="G50" t="str">
-        <v>로얄동 리모델링 추진단지 수지구청역초역세권 입주협의</v>
+        <v>입주가,  샷시포함 올수리되고 깨끗함</v>
       </c>
       <c r="H50" t="str">
         <v>naver</v>
@@ -1948,22 +1948,22 @@
         <v>현대</v>
       </c>
       <c r="B60" t="str">
-        <v>9억 9,000</v>
+        <v>9억 5,000</v>
       </c>
       <c r="C60">
         <v>74</v>
       </c>
       <c r="D60" t="str">
-        <v>101동</v>
+        <v>103동</v>
       </c>
       <c r="E60" t="str">
-        <v>9/15</v>
+        <v>5/15</v>
       </c>
       <c r="F60" t="str">
-        <v>남동향</v>
+        <v>남서향</v>
       </c>
       <c r="G60" t="str">
-        <v>로열동  로열층 내부수리 했었던 집 수지구청역 도보5분 초역세권</v>
+        <v>기본, 정상입주협의, 수지구청역 초역세권, 명문학군,편의시설다양</v>
       </c>
       <c r="H60" t="str">
         <v>naver</v>
@@ -2000,22 +2000,22 @@
         <v>현대</v>
       </c>
       <c r="B62" t="str">
-        <v>9억 5,000</v>
+        <v>9억 9,000</v>
       </c>
       <c r="C62">
         <v>74</v>
       </c>
       <c r="D62" t="str">
-        <v>103동</v>
+        <v>101동</v>
       </c>
       <c r="E62" t="str">
-        <v>5/15</v>
+        <v>9/15</v>
       </c>
       <c r="F62" t="str">
-        <v>남서향</v>
+        <v>남동향</v>
       </c>
       <c r="G62" t="str">
-        <v>기본, 정상입주협의, 수지구청역 초역세권, 명문학군,편의시설다양</v>
+        <v>로열동  로열층 내부수리 했었던 집 수지구청역 도보5분 초역세권</v>
       </c>
       <c r="H62" t="str">
         <v>naver</v>
@@ -2026,22 +2026,22 @@
         <v>현대</v>
       </c>
       <c r="B63" t="str">
-        <v>11억 8,000</v>
+        <v>12억</v>
       </c>
       <c r="C63">
         <v>104</v>
       </c>
       <c r="D63" t="str">
-        <v>102동</v>
+        <v>105동</v>
       </c>
       <c r="E63" t="str">
-        <v>6/15</v>
+        <v>9/15</v>
       </c>
       <c r="F63" t="str">
         <v>남동향</v>
       </c>
       <c r="G63" t="str">
-        <v>내부수리, 수지구청역 초역세권, 명문학군, 로얄층, 편의시설다양</v>
+        <v>로열동 내부수리 전망트여 시원해요  신분당선도보5분  생활인프라최고</v>
       </c>
       <c r="H63" t="str">
         <v>naver</v>
@@ -2052,22 +2052,22 @@
         <v>현대</v>
       </c>
       <c r="B64" t="str">
-        <v>11억 8,000</v>
+        <v>12억</v>
       </c>
       <c r="C64">
         <v>104</v>
       </c>
       <c r="D64" t="str">
-        <v>104동</v>
+        <v>111동</v>
       </c>
       <c r="E64" t="str">
-        <v>7/15</v>
+        <v>8/15</v>
       </c>
       <c r="F64" t="str">
-        <v>남서향</v>
+        <v>남동향</v>
       </c>
       <c r="G64" t="str">
-        <v>입주급매 앞 뒤 트여 바람 잘 통하고 밝은 집  살기 좋아요</v>
+        <v>입주협의, 부분수리된 집, 수지구청역 가까운 동, 로얄동</v>
       </c>
       <c r="H64" t="str">
         <v>naver</v>
@@ -2078,22 +2078,22 @@
         <v>현대</v>
       </c>
       <c r="B65" t="str">
-        <v>12억</v>
+        <v>11억 9,000</v>
       </c>
       <c r="C65">
         <v>104</v>
       </c>
       <c r="D65" t="str">
-        <v>111동</v>
+        <v>106동</v>
       </c>
       <c r="E65" t="str">
-        <v>8/15</v>
+        <v>12/15</v>
       </c>
       <c r="F65" t="str">
         <v>남동향</v>
       </c>
       <c r="G65" t="str">
-        <v>입주협의, 부분수리된 집, 수지구청역 가까운 동, 로얄동</v>
+        <v>수리깨끗, 수지구청역 초역세권, 명문학군,로얄동층, 편의시설다양</v>
       </c>
       <c r="H65" t="str">
         <v>naver</v>
@@ -2104,22 +2104,22 @@
         <v>현대</v>
       </c>
       <c r="B66" t="str">
-        <v>12억</v>
+        <v>11억 8,000</v>
       </c>
       <c r="C66">
         <v>104</v>
       </c>
       <c r="D66" t="str">
-        <v>105동</v>
+        <v>104동</v>
       </c>
       <c r="E66" t="str">
-        <v>9/15</v>
+        <v>7/15</v>
       </c>
       <c r="F66" t="str">
-        <v>남동향</v>
+        <v>남서향</v>
       </c>
       <c r="G66" t="str">
-        <v>로열동 내부수리 전망트여 시원해요  신분당선도보5분  생활인프라최고</v>
+        <v>입주급매 앞 뒤 트여 바람 잘 통하고 밝은 집  살기 좋아요</v>
       </c>
       <c r="H66" t="str">
         <v>naver</v>
@@ -2130,22 +2130,22 @@
         <v>현대</v>
       </c>
       <c r="B67" t="str">
-        <v>12억</v>
+        <v>11억 8,000</v>
       </c>
       <c r="C67">
         <v>104</v>
       </c>
       <c r="D67" t="str">
-        <v>109동</v>
+        <v>102동</v>
       </c>
       <c r="E67" t="str">
-        <v>2/15</v>
+        <v>6/15</v>
       </c>
       <c r="F67" t="str">
         <v>남동향</v>
       </c>
       <c r="G67" t="str">
-        <v>입주가능  중간샷시설치 중문설치 내부수리  로열동 저층 햇살 좋아요</v>
+        <v>내부수리, 수지구청역 초역세권, 명문학군, 로얄층, 편의시설다양</v>
       </c>
       <c r="H67" t="str">
         <v>naver</v>
@@ -2156,22 +2156,22 @@
         <v>현대</v>
       </c>
       <c r="B68" t="str">
-        <v>11억 9,000</v>
+        <v>12억</v>
       </c>
       <c r="C68">
         <v>104</v>
       </c>
       <c r="D68" t="str">
-        <v>106동</v>
+        <v>109동</v>
       </c>
       <c r="E68" t="str">
-        <v>12/15</v>
+        <v>2/15</v>
       </c>
       <c r="F68" t="str">
         <v>남동향</v>
       </c>
       <c r="G68" t="str">
-        <v>수리깨끗, 수지구청역 초역세권, 명문학군,로얄동층, 편의시설다양</v>
+        <v>입주가능  중간샷시설치 중문설치 내부수리  로열동 저층 햇살 좋아요</v>
       </c>
       <c r="H68" t="str">
         <v>naver</v>
@@ -2286,22 +2286,22 @@
         <v>현대</v>
       </c>
       <c r="B73" t="str">
-        <v>12억 5,000</v>
+        <v>11억</v>
       </c>
       <c r="C73">
         <v>104</v>
       </c>
       <c r="D73" t="str">
-        <v>106동</v>
+        <v>109동</v>
       </c>
       <c r="E73" t="str">
-        <v>2/15</v>
+        <v>1/15</v>
       </c>
       <c r="F73" t="str">
         <v>남동향</v>
       </c>
       <c r="G73" t="str">
-        <v>깨끗함, 기본상태, 8월말 입주가능</v>
+        <v>입주추천.샷시.화장실등 전체 올수리.역세권</v>
       </c>
       <c r="H73" t="str">
         <v>naver</v>
@@ -2312,22 +2312,22 @@
         <v>현대</v>
       </c>
       <c r="B74" t="str">
-        <v>9억 7,000</v>
+        <v>12억 5,000</v>
       </c>
       <c r="C74">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="D74" t="str">
-        <v>101동</v>
+        <v>106동</v>
       </c>
       <c r="E74" t="str">
-        <v>9/15</v>
+        <v>2/15</v>
       </c>
       <c r="F74" t="str">
         <v>남동향</v>
       </c>
       <c r="G74" t="str">
-        <v>예전수리된집, 10월말 입주가능</v>
+        <v>깨끗함, 기본상태, 8월말 입주가능</v>
       </c>
       <c r="H74" t="str">
         <v>naver</v>
@@ -2338,22 +2338,22 @@
         <v>현대</v>
       </c>
       <c r="B75" t="str">
-        <v>11억</v>
+        <v>9억 7,000</v>
       </c>
       <c r="C75">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="D75" t="str">
-        <v>109동</v>
+        <v>101동</v>
       </c>
       <c r="E75" t="str">
-        <v>1/15</v>
+        <v>9/15</v>
       </c>
       <c r="F75" t="str">
         <v>남동향</v>
       </c>
       <c r="G75" t="str">
-        <v>입주추천.샷시.화장실등 전체 올수리.역세권</v>
+        <v>예전수리된집, 10월말 입주가능</v>
       </c>
       <c r="H75" t="str">
         <v>naver</v>
@@ -2364,22 +2364,22 @@
         <v>현대</v>
       </c>
       <c r="B76" t="str">
-        <v>12억</v>
+        <v>11억</v>
       </c>
       <c r="C76">
         <v>104</v>
       </c>
       <c r="D76" t="str">
-        <v>112동</v>
+        <v>104동</v>
       </c>
       <c r="E76" t="str">
-        <v>3/15</v>
+        <v>1/15</v>
       </c>
       <c r="F76" t="str">
-        <v>남동향</v>
+        <v>남서향</v>
       </c>
       <c r="G76" t="str">
-        <v>정상입주 입주일협의 수지구청역 초역세권</v>
+        <v>세안고, 아이 키우기 좋아요. 동간 거리 넓고 조용한 동</v>
       </c>
       <c r="H76" t="str">
         <v>naver</v>
@@ -2390,22 +2390,22 @@
         <v>현대</v>
       </c>
       <c r="B77" t="str">
-        <v>11억</v>
+        <v>12억</v>
       </c>
       <c r="C77">
         <v>104</v>
       </c>
       <c r="D77" t="str">
-        <v>104동</v>
+        <v>112동</v>
       </c>
       <c r="E77" t="str">
-        <v>1/15</v>
+        <v>3/15</v>
       </c>
       <c r="F77" t="str">
-        <v>남서향</v>
+        <v>남동향</v>
       </c>
       <c r="G77" t="str">
-        <v>세안고, 아이 키우기 좋아요. 동간 거리 넓고 조용한 동</v>
+        <v>정상입주 입주일협의 수지구청역 초역세권</v>
       </c>
       <c r="H77" t="str">
         <v>naver</v>
@@ -2812,16 +2812,16 @@
         <v>78</v>
       </c>
       <c r="D93" t="str">
-        <v>103동</v>
+        <v>104동</v>
       </c>
       <c r="E93" t="str">
-        <v>5/17</v>
+        <v>12/17</v>
       </c>
       <c r="F93" t="str">
         <v>남동향</v>
       </c>
       <c r="G93" t="str">
-        <v>협의가능 투자가치굿, 도보역세권, 리모델링단지</v>
+        <v>R2, 주인거주, 올수리, 리모델링사업진행중</v>
       </c>
       <c r="H93" t="str">
         <v>naver</v>
@@ -2832,22 +2832,22 @@
         <v>동부</v>
       </c>
       <c r="B94" t="str">
-        <v>8억 2,000</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C94">
         <v>78</v>
       </c>
       <c r="D94" t="str">
-        <v>102동</v>
+        <v>103동</v>
       </c>
       <c r="E94" t="str">
-        <v>8/17</v>
+        <v>5/17</v>
       </c>
       <c r="F94" t="str">
         <v>남동향</v>
       </c>
       <c r="G94" t="str">
-        <v>입주급매 신분당선도보8분 내부수리됨 아파트뒤 도서관 소아병동입점</v>
+        <v>협의가능 투자가치굿, 도보역세권, 리모델링단지</v>
       </c>
       <c r="H94" t="str">
         <v>naver</v>
@@ -2858,22 +2858,22 @@
         <v>동부</v>
       </c>
       <c r="B95" t="str">
-        <v>8억 5,000</v>
+        <v>8억 2,000</v>
       </c>
       <c r="C95">
         <v>78</v>
       </c>
       <c r="D95" t="str">
-        <v>101동</v>
+        <v>102동</v>
       </c>
       <c r="E95" t="str">
-        <v>2/17</v>
+        <v>8/17</v>
       </c>
       <c r="F95" t="str">
         <v>남동향</v>
       </c>
       <c r="G95" t="str">
-        <v>방3 특올수리 거실확장 리모델링 진행중</v>
+        <v>입주급매 신분당선도보8분 내부수리됨 아파트뒤 도서관 소아병동입점</v>
       </c>
       <c r="H95" t="str">
         <v>naver</v>
@@ -2884,7 +2884,7 @@
         <v>동부</v>
       </c>
       <c r="B96" t="str">
-        <v>9억 2,000</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C96">
         <v>78</v>
@@ -2893,13 +2893,13 @@
         <v>105동</v>
       </c>
       <c r="E96" t="str">
-        <v>11/17</v>
+        <v>17/17</v>
       </c>
       <c r="F96" t="str">
         <v>남동향</v>
       </c>
       <c r="G96" t="str">
-        <v>R3, 주인거주,올수리,리모델링사업진행중</v>
+        <v xml:space="preserve">방3 리모델링 사업 진행중 입주일협의 </v>
       </c>
       <c r="H96" t="str">
         <v>naver</v>
@@ -2910,13 +2910,13 @@
         <v>동부</v>
       </c>
       <c r="B97" t="str">
-        <v>8억 8,000</v>
+        <v>9억 8,000</v>
       </c>
       <c r="C97">
         <v>78</v>
       </c>
       <c r="D97" t="str">
-        <v>103동</v>
+        <v>102동</v>
       </c>
       <c r="E97" t="str">
         <v>17/17</v>
@@ -2925,7 +2925,7 @@
         <v>남동향</v>
       </c>
       <c r="G97" t="str">
-        <v>최근 샷시포함 특올수리, 거실확장, 신혼부부 거주중</v>
+        <v>R2, 주인거주, 특올수리, 리모델링사업진행중</v>
       </c>
       <c r="H97" t="str">
         <v>naver</v>
@@ -2936,22 +2936,22 @@
         <v>동부</v>
       </c>
       <c r="B98" t="str">
-        <v>8억 5,000</v>
+        <v>8억 7,000</v>
       </c>
       <c r="C98">
         <v>78</v>
       </c>
       <c r="D98" t="str">
-        <v>104동</v>
+        <v>106동</v>
       </c>
       <c r="E98" t="str">
-        <v>12/17</v>
+        <v>2/17</v>
       </c>
       <c r="F98" t="str">
         <v>남동향</v>
       </c>
       <c r="G98" t="str">
-        <v>R2, 주인거주, 올수리, 리모델링사업진행중</v>
+        <v>방3, 거실확장 및 특올수리, 집상태 최고</v>
       </c>
       <c r="H98" t="str">
         <v>naver</v>
@@ -2962,22 +2962,22 @@
         <v>동부</v>
       </c>
       <c r="B99" t="str">
-        <v>8억 5,000</v>
+        <v>10억</v>
       </c>
       <c r="C99">
         <v>78</v>
       </c>
       <c r="D99" t="str">
-        <v>104동</v>
+        <v>106동</v>
       </c>
       <c r="E99" t="str">
-        <v>2/17</v>
+        <v>8/17</v>
       </c>
       <c r="F99" t="str">
         <v>남동향</v>
       </c>
       <c r="G99" t="str">
-        <v>R2, 주인거주, 올수리, 리모델링사업진행중</v>
+        <v>협의가능, 투자가치굿, 로얄동, 채광좋음</v>
       </c>
       <c r="H99" t="str">
         <v>naver</v>
@@ -2988,13 +2988,13 @@
         <v>동부</v>
       </c>
       <c r="B100" t="str">
-        <v>9억 8,000</v>
+        <v>8억 8,000</v>
       </c>
       <c r="C100">
         <v>78</v>
       </c>
       <c r="D100" t="str">
-        <v>102동</v>
+        <v>103동</v>
       </c>
       <c r="E100" t="str">
         <v>17/17</v>
@@ -3003,7 +3003,7 @@
         <v>남동향</v>
       </c>
       <c r="G100" t="str">
-        <v>R2, 주인거주, 특올수리, 리모델링사업진행중</v>
+        <v>최근 샷시포함 특올수리, 거실확장, 신혼부부 거주중</v>
       </c>
       <c r="H100" t="str">
         <v>naver</v>
@@ -3014,22 +3014,22 @@
         <v>동부</v>
       </c>
       <c r="B101" t="str">
-        <v>10억</v>
+        <v>9억</v>
       </c>
       <c r="C101">
         <v>78</v>
       </c>
       <c r="D101" t="str">
-        <v>106동</v>
+        <v>101동</v>
       </c>
       <c r="E101" t="str">
-        <v>8/17</v>
+        <v>6/17</v>
       </c>
       <c r="F101" t="str">
         <v>남동향</v>
       </c>
       <c r="G101" t="str">
-        <v>협의가능, 투자가치굿, 로얄동, 채광좋음</v>
+        <v>방3 리모델링 입주협의</v>
       </c>
       <c r="H101" t="str">
         <v>naver</v>
@@ -3040,13 +3040,13 @@
         <v>동부</v>
       </c>
       <c r="B102" t="str">
-        <v>8억 7,000</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C102">
         <v>78</v>
       </c>
       <c r="D102" t="str">
-        <v>106동</v>
+        <v>101동</v>
       </c>
       <c r="E102" t="str">
         <v>2/17</v>
@@ -3055,7 +3055,7 @@
         <v>남동향</v>
       </c>
       <c r="G102" t="str">
-        <v>방3, 거실확장 및 특올수리, 집상태 최고</v>
+        <v>방3 특올수리 거실확장 리모델링 진행중</v>
       </c>
       <c r="H102" t="str">
         <v>naver</v>
@@ -3072,16 +3072,16 @@
         <v>78</v>
       </c>
       <c r="D103" t="str">
-        <v>105동</v>
+        <v>104동</v>
       </c>
       <c r="E103" t="str">
-        <v>17/17</v>
+        <v>2/17</v>
       </c>
       <c r="F103" t="str">
         <v>남동향</v>
       </c>
       <c r="G103" t="str">
-        <v xml:space="preserve">방3 리모델링 사업 진행중 입주일협의 </v>
+        <v>R2, 주인거주, 올수리, 리모델링사업진행중</v>
       </c>
       <c r="H103" t="str">
         <v>naver</v>
@@ -3092,22 +3092,22 @@
         <v>동부</v>
       </c>
       <c r="B104" t="str">
-        <v>9억</v>
+        <v>9억 2,000</v>
       </c>
       <c r="C104">
         <v>78</v>
       </c>
       <c r="D104" t="str">
-        <v>101동</v>
+        <v>105동</v>
       </c>
       <c r="E104" t="str">
-        <v>6/17</v>
+        <v>11/17</v>
       </c>
       <c r="F104" t="str">
         <v>남동향</v>
       </c>
       <c r="G104" t="str">
-        <v>방3 리모델링 입주협의</v>
+        <v>R3, 주인거주,올수리,리모델링사업진행중</v>
       </c>
       <c r="H104" t="str">
         <v>naver</v>
@@ -3118,22 +3118,22 @@
         <v>동부</v>
       </c>
       <c r="B105" t="str">
-        <v>8억 7,000</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C105">
         <v>78</v>
       </c>
       <c r="D105" t="str">
-        <v>106동</v>
+        <v>103동</v>
       </c>
       <c r="E105" t="str">
-        <v>12/17</v>
+        <v>16/17</v>
       </c>
       <c r="F105" t="str">
         <v>남동향</v>
       </c>
       <c r="G105" t="str">
-        <v>방3화1, 계단식, 로얄동, 채광좋음</v>
+        <v>R2, 계단식,주인거주,로얄층,리모델링추진중</v>
       </c>
       <c r="H105" t="str">
         <v>naver</v>
@@ -3144,7 +3144,7 @@
         <v>동부</v>
       </c>
       <c r="B106" t="str">
-        <v>8억 7,000</v>
+        <v>8억 8,000</v>
       </c>
       <c r="C106">
         <v>78</v>
@@ -3153,13 +3153,13 @@
         <v>106동</v>
       </c>
       <c r="E106" t="str">
-        <v>11/17</v>
+        <v>9/17</v>
       </c>
       <c r="F106" t="str">
         <v>남동향</v>
       </c>
       <c r="G106" t="str">
-        <v>R3, 계단식,주인거주,올수리,리모델링추진중</v>
+        <v>R3, 계단식,주인거주,확장 특올수리,리모델링추진중</v>
       </c>
       <c r="H106" t="str">
         <v>naver</v>
@@ -3176,16 +3176,16 @@
         <v>78</v>
       </c>
       <c r="D107" t="str">
-        <v>101동</v>
+        <v>106동</v>
       </c>
       <c r="E107" t="str">
-        <v>5/17</v>
+        <v>8/17</v>
       </c>
       <c r="F107" t="str">
         <v>남동향</v>
       </c>
       <c r="G107" t="str">
-        <v>R3, 거실 방확장 올수리, 리모델링추진중</v>
+        <v>R3, 로얄층, 올수리,세안고,리모델링추진중</v>
       </c>
       <c r="H107" t="str">
         <v>naver</v>
@@ -3202,16 +3202,16 @@
         <v>78</v>
       </c>
       <c r="D108" t="str">
-        <v>106동</v>
+        <v>101동</v>
       </c>
       <c r="E108" t="str">
-        <v>8/17</v>
+        <v>5/17</v>
       </c>
       <c r="F108" t="str">
         <v>남동향</v>
       </c>
       <c r="G108" t="str">
-        <v>R3, 로얄층, 올수리,세안고,리모델링추진중</v>
+        <v>R3, 거실 방확장 올수리, 리모델링추진중</v>
       </c>
       <c r="H108" t="str">
         <v>naver</v>
@@ -3222,22 +3222,22 @@
         <v>동부</v>
       </c>
       <c r="B109" t="str">
-        <v>7억 5,000</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C109">
         <v>78</v>
       </c>
       <c r="D109" t="str">
-        <v>104동</v>
+        <v>106동</v>
       </c>
       <c r="E109" t="str">
-        <v>1/17</v>
+        <v>15/17</v>
       </c>
       <c r="F109" t="str">
         <v>남동향</v>
       </c>
       <c r="G109" t="str">
-        <v>입주협의  부분수리  방2  리모추진중  초중고 도서관 역세권 메디칼센터</v>
+        <v>R3, 계단식,주인거주, 로얄층, 리모델링추진중</v>
       </c>
       <c r="H109" t="str">
         <v>naver</v>
@@ -3248,22 +3248,22 @@
         <v>동부</v>
       </c>
       <c r="B110" t="str">
-        <v>8억 5,000</v>
+        <v>8억 7,000</v>
       </c>
       <c r="C110">
         <v>78</v>
       </c>
       <c r="D110" t="str">
-        <v>103동</v>
+        <v>106동</v>
       </c>
       <c r="E110" t="str">
-        <v>16/17</v>
+        <v>12/17</v>
       </c>
       <c r="F110" t="str">
         <v>남동향</v>
       </c>
       <c r="G110" t="str">
-        <v>R2, 계단식,주인거주,로얄층,리모델링추진중</v>
+        <v>방3화1, 계단식, 로얄동, 채광좋음</v>
       </c>
       <c r="H110" t="str">
         <v>naver</v>
@@ -3274,22 +3274,22 @@
         <v>동부</v>
       </c>
       <c r="B111" t="str">
-        <v>8억 8,000</v>
+        <v>7억 5,000</v>
       </c>
       <c r="C111">
         <v>78</v>
       </c>
       <c r="D111" t="str">
-        <v>106동</v>
+        <v>104동</v>
       </c>
       <c r="E111" t="str">
-        <v>9/17</v>
+        <v>1/17</v>
       </c>
       <c r="F111" t="str">
         <v>남동향</v>
       </c>
       <c r="G111" t="str">
-        <v>R3, 계단식,주인거주,확장 특올수리,리모델링추진중</v>
+        <v>입주협의  부분수리  방2  리모추진중  초중고 도서관 역세권 메디칼센터</v>
       </c>
       <c r="H111" t="str">
         <v>naver</v>
@@ -3300,7 +3300,7 @@
         <v>동부</v>
       </c>
       <c r="B112" t="str">
-        <v>8억 5,000</v>
+        <v>8억 7,000</v>
       </c>
       <c r="C112">
         <v>78</v>
@@ -3309,13 +3309,13 @@
         <v>106동</v>
       </c>
       <c r="E112" t="str">
-        <v>15/17</v>
+        <v>11/17</v>
       </c>
       <c r="F112" t="str">
         <v>남동향</v>
       </c>
       <c r="G112" t="str">
-        <v>R3, 계단식,주인거주, 로얄층, 리모델링추진중</v>
+        <v>R3, 계단식,주인거주,올수리,리모델링추진중</v>
       </c>
       <c r="H112" t="str">
         <v>naver</v>
@@ -3326,22 +3326,22 @@
         <v>동부</v>
       </c>
       <c r="B113" t="str">
-        <v>9억</v>
+        <v>9억 2,000</v>
       </c>
       <c r="C113">
         <v>78</v>
       </c>
       <c r="D113" t="str">
-        <v>102동</v>
+        <v>101동</v>
       </c>
       <c r="E113" t="str">
-        <v>6/17</v>
+        <v>10/17</v>
       </c>
       <c r="F113" t="str">
         <v>남동향</v>
       </c>
       <c r="G113" t="str">
-        <v>방2화1,  도보역세권, 채광좋음, 수리됨</v>
+        <v>방3화1, 채광좋음, 도보역세권, 일정등협의가능</v>
       </c>
       <c r="H113" t="str">
         <v>naver</v>
@@ -3410,16 +3410,16 @@
         <v>78</v>
       </c>
       <c r="D116" t="str">
-        <v>105동</v>
+        <v>102동</v>
       </c>
       <c r="E116" t="str">
-        <v>7/17</v>
+        <v>6/17</v>
       </c>
       <c r="F116" t="str">
         <v>남동향</v>
       </c>
       <c r="G116" t="str">
-        <v>방3화1, 계단식, 방확장, 채광좋음, 도보역세권</v>
+        <v>방2화1,  도보역세권, 채광좋음, 수리됨</v>
       </c>
       <c r="H116" t="str">
         <v>naver</v>
@@ -3439,13 +3439,13 @@
         <v>101동</v>
       </c>
       <c r="E117" t="str">
-        <v>10/17</v>
+        <v>8/17</v>
       </c>
       <c r="F117" t="str">
         <v>남동향</v>
       </c>
       <c r="G117" t="str">
-        <v>방3화1, 채광좋음, 도보역세권, 일정등협의가능</v>
+        <v>방3, 계단식, 샷시포함올수리, 채광좋음</v>
       </c>
       <c r="H117" t="str">
         <v>naver</v>
@@ -3456,22 +3456,22 @@
         <v>동부</v>
       </c>
       <c r="B118" t="str">
-        <v>9억 2,000</v>
+        <v>9억</v>
       </c>
       <c r="C118">
         <v>78</v>
       </c>
       <c r="D118" t="str">
-        <v>101동</v>
+        <v>105동</v>
       </c>
       <c r="E118" t="str">
-        <v>8/17</v>
+        <v>7/17</v>
       </c>
       <c r="F118" t="str">
         <v>남동향</v>
       </c>
       <c r="G118" t="str">
-        <v>방3, 계단식, 샷시포함올수리, 채광좋음</v>
+        <v>방3화1, 계단식, 방확장, 채광좋음, 도보역세권</v>
       </c>
       <c r="H118" t="str">
         <v>naver</v>
@@ -3534,22 +3534,22 @@
         <v>동부</v>
       </c>
       <c r="B121" t="str">
-        <v>8억 3,000</v>
+        <v>9억 3,000</v>
       </c>
       <c r="C121">
         <v>78</v>
       </c>
       <c r="D121" t="str">
-        <v>105동</v>
+        <v>101동</v>
       </c>
       <c r="E121" t="str">
-        <v>중/17</v>
+        <v>13/17</v>
       </c>
       <c r="F121" t="str">
         <v>남동향</v>
       </c>
       <c r="G121" t="str">
-        <v>꼭팔아요 급매 입주협의 방3  특올수리  초중고 역세권 선호하는동 강추</v>
+        <v>협의가능 투자가치굿, 우수인프라, 도보역세권</v>
       </c>
       <c r="H121" t="str">
         <v>naver</v>
@@ -3560,22 +3560,22 @@
         <v>동부</v>
       </c>
       <c r="B122" t="str">
-        <v>9억 3,000</v>
+        <v>8억 3,000</v>
       </c>
       <c r="C122">
         <v>78</v>
       </c>
       <c r="D122" t="str">
-        <v>101동</v>
+        <v>105동</v>
       </c>
       <c r="E122" t="str">
-        <v>13/17</v>
+        <v>중/17</v>
       </c>
       <c r="F122" t="str">
         <v>남동향</v>
       </c>
       <c r="G122" t="str">
-        <v>협의가능 투자가치굿, 우수인프라, 도보역세권</v>
+        <v>꼭팔아요 급매 입주협의 방3  특올수리  초중고 역세권 선호하는동 강추</v>
       </c>
       <c r="H122" t="str">
         <v>naver</v>
@@ -3592,16 +3592,16 @@
         <v>78</v>
       </c>
       <c r="D123" t="str">
-        <v>105동</v>
+        <v>101동</v>
       </c>
       <c r="E123" t="str">
-        <v>고/17</v>
+        <v>중/17</v>
       </c>
       <c r="F123" t="str">
         <v>남동향</v>
       </c>
       <c r="G123" t="str">
-        <v>샷시 제외 특올수리이며 입주 가능하고 리모델링 추진 단지임</v>
+        <v>방3,주인거주,리모델링 이주확정</v>
       </c>
       <c r="H123" t="str">
         <v>naver</v>
@@ -3612,22 +3612,22 @@
         <v>동부</v>
       </c>
       <c r="B124" t="str">
-        <v>8억 5,000</v>
+        <v>8억 7,000</v>
       </c>
       <c r="C124">
         <v>78</v>
       </c>
       <c r="D124" t="str">
-        <v>105동</v>
+        <v>103동</v>
       </c>
       <c r="E124" t="str">
-        <v>중/17</v>
+        <v>고/17</v>
       </c>
       <c r="F124" t="str">
         <v>남동향</v>
       </c>
       <c r="G124" t="str">
-        <v>입주가능 화장실포함올수리 방3개 수지구청역도보권및도서관인접</v>
+        <v>방2화1, 계단식, 채광좋음, 도보역세권</v>
       </c>
       <c r="H124" t="str">
         <v>naver</v>
@@ -3638,22 +3638,22 @@
         <v>동부</v>
       </c>
       <c r="B125" t="str">
-        <v>8억 7,000</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C125">
         <v>78</v>
       </c>
       <c r="D125" t="str">
-        <v>103동</v>
+        <v>105동</v>
       </c>
       <c r="E125" t="str">
-        <v>고/17</v>
+        <v>중/17</v>
       </c>
       <c r="F125" t="str">
         <v>남동향</v>
       </c>
       <c r="G125" t="str">
-        <v>방2화1, 계단식, 채광좋음, 도보역세권</v>
+        <v>입주가능 화장실포함올수리 방3개 수지구청역도보권및도서관인접</v>
       </c>
       <c r="H125" t="str">
         <v>naver</v>
@@ -3670,16 +3670,16 @@
         <v>78</v>
       </c>
       <c r="D126" t="str">
-        <v>101동</v>
+        <v>105동</v>
       </c>
       <c r="E126" t="str">
-        <v>중/17</v>
+        <v>고/17</v>
       </c>
       <c r="F126" t="str">
         <v>남동향</v>
       </c>
       <c r="G126" t="str">
-        <v>방3,주인거주,리모델링 이주확정</v>
+        <v>샷시 제외 특올수리이며 입주 가능하고 리모델링 추진 단지임</v>
       </c>
       <c r="H126" t="str">
         <v>naver</v>
@@ -3690,13 +3690,13 @@
         <v>동부</v>
       </c>
       <c r="B127" t="str">
-        <v>8억 6,000</v>
+        <v>9억</v>
       </c>
       <c r="C127">
         <v>78</v>
       </c>
       <c r="D127" t="str">
-        <v>103동</v>
+        <v>102동</v>
       </c>
       <c r="E127" t="str">
         <v>중/17</v>
@@ -3705,7 +3705,7 @@
         <v>남동향</v>
       </c>
       <c r="G127" t="str">
-        <v>방2화1, 로얄동로얄층, 올수리, 채광좋음</v>
+        <v>방2화1, 채광좋음, 올수리, 도보역세권</v>
       </c>
       <c r="H127" t="str">
         <v>naver</v>
@@ -3716,22 +3716,22 @@
         <v>동부</v>
       </c>
       <c r="B128" t="str">
-        <v>9억</v>
+        <v>8억 6,000</v>
       </c>
       <c r="C128">
         <v>78</v>
       </c>
       <c r="D128" t="str">
-        <v>104동</v>
+        <v>103동</v>
       </c>
       <c r="E128" t="str">
-        <v>고/17</v>
+        <v>중/17</v>
       </c>
       <c r="F128" t="str">
         <v>남동향</v>
       </c>
       <c r="G128" t="str">
-        <v>올수리, 도보역세권, 일정 등 협의가능</v>
+        <v>방2화1, 로얄동로얄층, 올수리, 채광좋음</v>
       </c>
       <c r="H128" t="str">
         <v>naver</v>
@@ -3748,16 +3748,16 @@
         <v>78</v>
       </c>
       <c r="D129" t="str">
-        <v>102동</v>
+        <v>104동</v>
       </c>
       <c r="E129" t="str">
-        <v>중/17</v>
+        <v>고/17</v>
       </c>
       <c r="F129" t="str">
         <v>남동향</v>
       </c>
       <c r="G129" t="str">
-        <v>방2화1, 채광좋음, 올수리, 도보역세권</v>
+        <v>올수리, 도보역세권, 일정 등 협의가능</v>
       </c>
       <c r="H129" t="str">
         <v>naver</v>
@@ -3794,16 +3794,16 @@
         <v>동부</v>
       </c>
       <c r="B131" t="str">
-        <v>8억 5,000</v>
+        <v>9억</v>
       </c>
       <c r="C131">
         <v>78</v>
       </c>
       <c r="D131" t="str">
-        <v>104동</v>
+        <v>102동</v>
       </c>
       <c r="E131" t="str">
-        <v>5/17</v>
+        <v>16/17</v>
       </c>
       <c r="F131" t="str">
         <v>남동향</v>
@@ -3820,16 +3820,16 @@
         <v>동부</v>
       </c>
       <c r="B132" t="str">
-        <v>9억</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C132">
         <v>78</v>
       </c>
       <c r="D132" t="str">
-        <v>102동</v>
+        <v>104동</v>
       </c>
       <c r="E132" t="str">
-        <v>16/17</v>
+        <v>5/17</v>
       </c>
       <c r="F132" t="str">
         <v>남동향</v>
@@ -4034,16 +4034,16 @@
         <v>78</v>
       </c>
       <c r="D140" t="str">
-        <v>101동</v>
+        <v>102동</v>
       </c>
       <c r="E140" t="str">
-        <v>고/17</v>
+        <v>저/17</v>
       </c>
       <c r="F140" t="str">
         <v>남동향</v>
       </c>
       <c r="G140" t="str">
-        <v>방3 계단식,올수리,전망, 전철역세권</v>
+        <v>입주협의거실확장 샤시일부교체 리모추진중 역세권 초중고인접 도서관 메디컬외</v>
       </c>
       <c r="H140" t="str">
         <v>naver</v>
@@ -4054,22 +4054,22 @@
         <v>동부</v>
       </c>
       <c r="B141" t="str">
-        <v>9억</v>
+        <v>9억 3,000</v>
       </c>
       <c r="C141">
         <v>78</v>
       </c>
       <c r="D141" t="str">
-        <v>106동</v>
+        <v>105동</v>
       </c>
       <c r="E141" t="str">
-        <v>7/17</v>
+        <v>중/17</v>
       </c>
       <c r="F141" t="str">
         <v>남동향</v>
       </c>
       <c r="G141" t="str">
-        <v>방3 계단식,주인거주,로얄층,수리,전철역세권</v>
+        <v>입주협의 방3  최근올수리 초중고인접 도서관 메디칼센터 역세권 공원인접</v>
       </c>
       <c r="H141" t="str">
         <v>naver</v>
@@ -4086,16 +4086,16 @@
         <v>78</v>
       </c>
       <c r="D142" t="str">
-        <v>102동</v>
+        <v>101동</v>
       </c>
       <c r="E142" t="str">
-        <v>저/17</v>
+        <v>고/17</v>
       </c>
       <c r="F142" t="str">
         <v>남동향</v>
       </c>
       <c r="G142" t="str">
-        <v>입주협의거실확장 샤시일부교체 리모추진중 역세권 초중고인접 도서관 메디컬외</v>
+        <v>방3 계단식,올수리,전망, 전철역세권</v>
       </c>
       <c r="H142" t="str">
         <v>naver</v>
@@ -4106,22 +4106,22 @@
         <v>동부</v>
       </c>
       <c r="B143" t="str">
-        <v>9억 3,000</v>
+        <v>9억</v>
       </c>
       <c r="C143">
         <v>78</v>
       </c>
       <c r="D143" t="str">
-        <v>105동</v>
+        <v>106동</v>
       </c>
       <c r="E143" t="str">
-        <v>중/17</v>
+        <v>7/17</v>
       </c>
       <c r="F143" t="str">
         <v>남동향</v>
       </c>
       <c r="G143" t="str">
-        <v>입주협의 방3  최근올수리 초중고인접 도서관 메디칼센터 역세권 공원인접</v>
+        <v>방3 계단식,주인거주,로얄층,수리,전철역세권</v>
       </c>
       <c r="H143" t="str">
         <v>naver</v>
@@ -4132,22 +4132,22 @@
         <v>동부</v>
       </c>
       <c r="B144" t="str">
-        <v>8억 5,000</v>
+        <v>8억 2,000</v>
       </c>
       <c r="C144">
         <v>78</v>
       </c>
       <c r="D144" t="str">
-        <v>104동</v>
+        <v>103동</v>
       </c>
       <c r="E144" t="str">
-        <v>3/17</v>
+        <v>17/17</v>
       </c>
       <c r="F144" t="str">
         <v>남동향</v>
       </c>
       <c r="G144" t="str">
-        <v>깨끗함, 기본상태, 주인거주 정상입주</v>
+        <v>깨끗함, 주인거주</v>
       </c>
       <c r="H144" t="str">
         <v>naver</v>
@@ -4158,22 +4158,22 @@
         <v>동부</v>
       </c>
       <c r="B145" t="str">
-        <v>8억 2,000</v>
+        <v>8억 5,000</v>
       </c>
       <c r="C145">
         <v>78</v>
       </c>
       <c r="D145" t="str">
-        <v>103동</v>
+        <v>104동</v>
       </c>
       <c r="E145" t="str">
-        <v>17/17</v>
+        <v>3/17</v>
       </c>
       <c r="F145" t="str">
         <v>남동향</v>
       </c>
       <c r="G145" t="str">
-        <v>깨끗함, 주인거주</v>
+        <v>깨끗함, 기본상태, 주인거주 정상입주</v>
       </c>
       <c r="H145" t="str">
         <v>naver</v>
@@ -4883,9 +4883,2193 @@
         <v>naver</v>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B173" t="str">
+        <v>10억 9,000</v>
+      </c>
+      <c r="C173">
+        <v>122</v>
+      </c>
+      <c r="D173" t="str">
+        <v>104동</v>
+      </c>
+      <c r="E173" t="str">
+        <v>23/25</v>
+      </c>
+      <c r="F173" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G173" t="str">
+        <v>역세권 단지 탁트인 전망의 엘베 연결 로얄동 입주 정상 협의</v>
+      </c>
+      <c r="H173" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B174" t="str">
+        <v>10억 9,000</v>
+      </c>
+      <c r="C174">
+        <v>122</v>
+      </c>
+      <c r="D174" t="str">
+        <v>103동</v>
+      </c>
+      <c r="E174" t="str">
+        <v>5/16</v>
+      </c>
+      <c r="F174" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G174" t="str">
+        <v>종일 밝은 정남향 올확장 깨끗관리 컨디션최고 동천역5분</v>
+      </c>
+      <c r="H174" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B175" t="str">
+        <v>10억 9,000</v>
+      </c>
+      <c r="C175">
+        <v>122</v>
+      </c>
+      <c r="D175" t="str">
+        <v>103동</v>
+      </c>
+      <c r="E175" t="str">
+        <v>중/16</v>
+      </c>
+      <c r="F175" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G175" t="str">
+        <v>동천역5분, 남향, 거실확장, 입주협의가능, 부분수리되어 깨끗함</v>
+      </c>
+      <c r="H175" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B176" t="str">
+        <v>10억 7,000</v>
+      </c>
+      <c r="C176">
+        <v>122</v>
+      </c>
+      <c r="D176" t="str">
+        <v>106동</v>
+      </c>
+      <c r="E176" t="str">
+        <v>저/16</v>
+      </c>
+      <c r="F176" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G176" t="str">
+        <v>동천역5분, 남향, 세안고매매, 올확장, 1층아님, 주차연결동</v>
+      </c>
+      <c r="H176" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B177" t="str">
+        <v>12억</v>
+      </c>
+      <c r="C177">
+        <v>122</v>
+      </c>
+      <c r="D177" t="str">
+        <v>101동</v>
+      </c>
+      <c r="E177" t="str">
+        <v>8/25</v>
+      </c>
+      <c r="F177" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G177" t="str">
+        <v>37. 신분당선동천역 화이트톤올수리 확트인뷰 해 잘드는집 정남향 입주협</v>
+      </c>
+      <c r="H177" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B178" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C178">
+        <v>122</v>
+      </c>
+      <c r="D178" t="str">
+        <v>104동</v>
+      </c>
+      <c r="E178" t="str">
+        <v>6/25</v>
+      </c>
+      <c r="F178" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G178" t="str">
+        <v>동천역5분, 남향, 주방,욕실,도배,장판,탄성 등 수리됨, 가격조정가</v>
+      </c>
+      <c r="H178" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B179" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C179">
+        <v>122</v>
+      </c>
+      <c r="D179" t="str">
+        <v>106동</v>
+      </c>
+      <c r="E179" t="str">
+        <v>고/16</v>
+      </c>
+      <c r="F179" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G179" t="str">
+        <v>동천역5분, 남향, 로열동, 주차연결, 입주협의가능, 수리기간드림</v>
+      </c>
+      <c r="H179" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B180" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C180">
+        <v>122</v>
+      </c>
+      <c r="D180" t="str">
+        <v>104동</v>
+      </c>
+      <c r="E180" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F180" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G180" t="str">
+        <v>동천역5분, 남향, 화이트수리, 비확장, 입주협의가능</v>
+      </c>
+      <c r="H180" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B181" t="str">
+        <v>11억 9,000</v>
+      </c>
+      <c r="C181">
+        <v>122</v>
+      </c>
+      <c r="D181" t="str">
+        <v>101동</v>
+      </c>
+      <c r="E181" t="str">
+        <v>저/25</v>
+      </c>
+      <c r="F181" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G181" t="str">
+        <v>H. 햇살가득 따뜻한 남향 올확장 화이트수리 관리최상 동천역</v>
+      </c>
+      <c r="H181" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B182" t="str">
+        <v>11억 5,000</v>
+      </c>
+      <c r="C182">
+        <v>122</v>
+      </c>
+      <c r="D182" t="str">
+        <v>105동</v>
+      </c>
+      <c r="E182" t="str">
+        <v>중/16</v>
+      </c>
+      <c r="F182" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G182" t="str">
+        <v>동천역5분, 남향, 전망굿, 로열동, 7월이후입주 협의가능</v>
+      </c>
+      <c r="H182" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B183" t="str">
+        <v>11억 7,000</v>
+      </c>
+      <c r="C183">
+        <v>122</v>
+      </c>
+      <c r="D183" t="str">
+        <v>107동</v>
+      </c>
+      <c r="E183" t="str">
+        <v>고/23</v>
+      </c>
+      <c r="F183" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G183" t="str">
+        <v>올수리. 2027.8월 임대안고, 전망좋은집, 동천역 도보3분</v>
+      </c>
+      <c r="H183" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B184" t="str">
+        <v>11억 7,000</v>
+      </c>
+      <c r="C184">
+        <v>122</v>
+      </c>
+      <c r="D184" t="str">
+        <v>107동</v>
+      </c>
+      <c r="E184" t="str">
+        <v>18/23</v>
+      </c>
+      <c r="F184" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G184" t="str">
+        <v>2027년 8월 월세안고, 전망이 좋은집, 동천역 도보5분거리,수리된집</v>
+      </c>
+      <c r="H184" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B185" t="str">
+        <v>10억 9,000</v>
+      </c>
+      <c r="C185" t="str">
+        <v>122</v>
+      </c>
+      <c r="D185" t="str">
+        <v>104동</v>
+      </c>
+      <c r="E185" t="str">
+        <v>고층</v>
+      </c>
+      <c r="F185" t="str">
+        <v/>
+      </c>
+      <c r="G185" t="str">
+        <v>햇살가득남향 특전망 로얄동 올수리 컨디션최고 엘베연결</v>
+      </c>
+      <c r="H185" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B186" t="str">
+        <v>10억 7,000</v>
+      </c>
+      <c r="C186" t="str">
+        <v>122</v>
+      </c>
+      <c r="D186" t="str">
+        <v>106동</v>
+      </c>
+      <c r="E186" t="str">
+        <v>고층</v>
+      </c>
+      <c r="F186" t="str">
+        <v/>
+      </c>
+      <c r="G186" t="str">
+        <v>동천역5분, 남향, 로열동, 주차연결, 입주협의가능, 수리기간드림</v>
+      </c>
+      <c r="H186" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>동천마을현대홈타운1차</v>
+      </c>
+      <c r="B187" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C187" t="str">
+        <v>122</v>
+      </c>
+      <c r="D187" t="str">
+        <v>104동</v>
+      </c>
+      <c r="E187" t="str">
+        <v>23층</v>
+      </c>
+      <c r="F187" t="str">
+        <v/>
+      </c>
+      <c r="G187" t="str">
+        <v>동천역5분, 남향, 전망굿, 부분수리, 주차연결동, 입주협의가능</v>
+      </c>
+      <c r="H187" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B188" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C188">
+        <v>122</v>
+      </c>
+      <c r="D188" t="str">
+        <v>204동</v>
+      </c>
+      <c r="E188" t="str">
+        <v>20/25</v>
+      </c>
+      <c r="F188" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G188" t="str">
+        <v>남향 조용한단지전망 햇볕짱 부분수리 싱크대,도기교체 세안고</v>
+      </c>
+      <c r="H188" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B189" t="str">
+        <v>10억</v>
+      </c>
+      <c r="C189">
+        <v>81</v>
+      </c>
+      <c r="D189" t="str">
+        <v>201동</v>
+      </c>
+      <c r="E189" t="str">
+        <v>5/25</v>
+      </c>
+      <c r="F189" t="str">
+        <v>동향</v>
+      </c>
+      <c r="G189" t="str">
+        <v>o.최근화이트특올수리.샤시교체. 트인전망시원함. 조용한입구동,신혼추천</v>
+      </c>
+      <c r="H189" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B190" t="str">
+        <v>10억 5,000</v>
+      </c>
+      <c r="C190">
+        <v>122</v>
+      </c>
+      <c r="D190" t="str">
+        <v>204동</v>
+      </c>
+      <c r="E190" t="str">
+        <v>6/25</v>
+      </c>
+      <c r="F190" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G190" t="str">
+        <v>따스한남향 조용한단지전망 동천역인접동 동천역세권 세안고</v>
+      </c>
+      <c r="H190" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B191" t="str">
+        <v>10억 3,000</v>
+      </c>
+      <c r="C191">
+        <v>122</v>
+      </c>
+      <c r="D191" t="str">
+        <v>204동</v>
+      </c>
+      <c r="E191" t="str">
+        <v>1/25</v>
+      </c>
+      <c r="F191" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G191" t="str">
+        <v>남향, 확장, 부분수리, 깨끗, 동천역가까운동, 입지좋은대단지</v>
+      </c>
+      <c r="H191" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B192" t="str">
+        <v>9억</v>
+      </c>
+      <c r="C192">
+        <v>81</v>
+      </c>
+      <c r="D192" t="str">
+        <v>201동</v>
+      </c>
+      <c r="E192" t="str">
+        <v>2/25</v>
+      </c>
+      <c r="F192" t="str">
+        <v>동향</v>
+      </c>
+      <c r="G192" t="str">
+        <v>대단지아파트 동천역근접동  기본형 9월초이후 교통편리</v>
+      </c>
+      <c r="H192" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B193" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C193">
+        <v>122</v>
+      </c>
+      <c r="D193" t="str">
+        <v>206동</v>
+      </c>
+      <c r="E193" t="str">
+        <v>중/25</v>
+      </c>
+      <c r="F193" t="str">
+        <v>동향</v>
+      </c>
+      <c r="G193" t="str">
+        <v>탁트인전망 채광굿 잘관리된집 동천역세권 입주협의</v>
+      </c>
+      <c r="H193" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B194" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C194">
+        <v>122</v>
+      </c>
+      <c r="D194" t="str">
+        <v>208동</v>
+      </c>
+      <c r="E194" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F194" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G194" t="str">
+        <v>남향 정상입주 로얄동 환상전망 채광굿 기본형</v>
+      </c>
+      <c r="H194" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B195" t="str">
+        <v>10억 6,000</v>
+      </c>
+      <c r="C195">
+        <v>122</v>
+      </c>
+      <c r="D195" t="str">
+        <v>206동</v>
+      </c>
+      <c r="E195" t="str">
+        <v>중/25</v>
+      </c>
+      <c r="F195" t="str">
+        <v>동향</v>
+      </c>
+      <c r="G195" t="str">
+        <v>올확장 시원한전망 관리가 잘된집  동천역세권 입주협의</v>
+      </c>
+      <c r="H195" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B196" t="str">
+        <v>11억 1,000</v>
+      </c>
+      <c r="C196">
+        <v>122</v>
+      </c>
+      <c r="D196" t="str">
+        <v>209동</v>
+      </c>
+      <c r="E196" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F196" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G196" t="str">
+        <v>따스한남향 로얄동 관리가잘된집 싱크대교체 채광굿 입주협의</v>
+      </c>
+      <c r="H196" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B197" t="str">
+        <v>9억 9,000</v>
+      </c>
+      <c r="C197">
+        <v>122</v>
+      </c>
+      <c r="D197" t="str">
+        <v>202동</v>
+      </c>
+      <c r="E197" t="str">
+        <v>저/24</v>
+      </c>
+      <c r="F197" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G197" t="str">
+        <v>H.햇살가득 따뜻한 남향 거실확장 부분수리 깔끔해요 동천역 세안고</v>
+      </c>
+      <c r="H197" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B198" t="str">
+        <v>10억 8,000</v>
+      </c>
+      <c r="C198">
+        <v>122</v>
+      </c>
+      <c r="D198" t="str">
+        <v>202동</v>
+      </c>
+      <c r="E198" t="str">
+        <v>고/24</v>
+      </c>
+      <c r="F198" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G198" t="str">
+        <v>H. 좋은집 밝고환한남향 관리최상 채광굿 주차편리 학세권 동천역</v>
+      </c>
+      <c r="H198" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B199" t="str">
+        <v>11억 5,000</v>
+      </c>
+      <c r="C199">
+        <v>122</v>
+      </c>
+      <c r="D199" t="str">
+        <v>207동</v>
+      </c>
+      <c r="E199" t="str">
+        <v>고/23</v>
+      </c>
+      <c r="F199" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G199" t="str">
+        <v>따스한남향 로얄동 관리가잘된집 화이트수리 채광굿 입주협의</v>
+      </c>
+      <c r="H199" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B200" t="str">
+        <v>11억 3,000</v>
+      </c>
+      <c r="C200">
+        <v>122</v>
+      </c>
+      <c r="D200" t="str">
+        <v>207동</v>
+      </c>
+      <c r="E200" t="str">
+        <v>6/23</v>
+      </c>
+      <c r="F200" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G200" t="str">
+        <v>로얄동 부분수리 채광굿 깔끔관리 정상입주</v>
+      </c>
+      <c r="H200" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B201" t="str">
+        <v>10억 5,000</v>
+      </c>
+      <c r="C201">
+        <v>122</v>
+      </c>
+      <c r="D201" t="str">
+        <v>204동</v>
+      </c>
+      <c r="E201" t="str">
+        <v>2/25</v>
+      </c>
+      <c r="F201" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G201" t="str">
+        <v>남향 확장형 화이트올수리 싱크대욕실ok   세안고</v>
+      </c>
+      <c r="H201" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>동천마을현대홈타운2차</v>
+      </c>
+      <c r="B202" t="str">
+        <v>11억 5,000</v>
+      </c>
+      <c r="C202">
+        <v>122</v>
+      </c>
+      <c r="D202" t="str">
+        <v>208동</v>
+      </c>
+      <c r="E202" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F202" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G202" t="str">
+        <v>로얄동층 굿라인 화이트올수리 환상전망 샷시교체 입주협의</v>
+      </c>
+      <c r="H202" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B203" t="str">
+        <v>11억 5,000</v>
+      </c>
+      <c r="C203">
+        <v>108</v>
+      </c>
+      <c r="D203" t="str">
+        <v>511동</v>
+      </c>
+      <c r="E203" t="str">
+        <v>22/24</v>
+      </c>
+      <c r="F203" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G203" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="H203" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B204" t="str">
+        <v>13억</v>
+      </c>
+      <c r="C204">
+        <v>108</v>
+      </c>
+      <c r="D204" t="str">
+        <v>514동</v>
+      </c>
+      <c r="E204" t="str">
+        <v>12/25</v>
+      </c>
+      <c r="F204" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G204" t="str">
+        <v>로얄동,프리미엄확장,트인전망,깔끔</v>
+      </c>
+      <c r="H204" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B205" t="str">
+        <v>12억 3,000</v>
+      </c>
+      <c r="C205">
+        <v>108</v>
+      </c>
+      <c r="D205" t="str">
+        <v>509동</v>
+      </c>
+      <c r="E205" t="str">
+        <v>20/25</v>
+      </c>
+      <c r="F205" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G205" t="str">
+        <v>입구동. 확장형.부분수리  컨디션 아주 좋음. 햇빛가득한 집.</v>
+      </c>
+      <c r="H205" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B206" t="str">
+        <v>12억 5,000</v>
+      </c>
+      <c r="C206">
+        <v>108</v>
+      </c>
+      <c r="D206" t="str">
+        <v>502동</v>
+      </c>
+      <c r="E206" t="str">
+        <v>10/21</v>
+      </c>
+      <c r="F206" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G206" t="str">
+        <v>앞트인 시원뷰.프리미엄확장.상태최상.입구동산책로근접,동천역도보권.생활편리</v>
+      </c>
+      <c r="H206" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B207" t="str">
+        <v>12억 2,000</v>
+      </c>
+      <c r="C207">
+        <v>108</v>
+      </c>
+      <c r="D207" t="str">
+        <v>514동</v>
+      </c>
+      <c r="E207" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F207" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G207" t="str">
+        <v>트인뷰,프리미엄확장형, 선호동,선호층,채광,환기좋음. 세안고</v>
+      </c>
+      <c r="H207" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B208" t="str">
+        <v>12억 5,000</v>
+      </c>
+      <c r="C208">
+        <v>108</v>
+      </c>
+      <c r="D208" t="str">
+        <v>509동</v>
+      </c>
+      <c r="E208" t="str">
+        <v>22/25</v>
+      </c>
+      <c r="F208" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G208" t="str">
+        <v>강추 눈부시게예쁜집 3년전특올수리올확장 시스템에어컨4대 동간거리넓은광장뷰</v>
+      </c>
+      <c r="H208" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B209" t="str">
+        <v>12억</v>
+      </c>
+      <c r="C209">
+        <v>108</v>
+      </c>
+      <c r="D209" t="str">
+        <v>514동</v>
+      </c>
+      <c r="E209" t="str">
+        <v>6/25</v>
+      </c>
+      <c r="F209" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G209" t="str">
+        <v>0318966776 수리됨입주협의전망짱</v>
+      </c>
+      <c r="H209" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B210" t="str">
+        <v>13억</v>
+      </c>
+      <c r="C210">
+        <v>108</v>
+      </c>
+      <c r="D210" t="str">
+        <v>512동</v>
+      </c>
+      <c r="E210" t="str">
+        <v>중/23</v>
+      </c>
+      <c r="F210" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G210" t="str">
+        <v>o.최근특올수리,올확장,화이트톤,탁트인전망,최로얄동층,상태최상,정상입주</v>
+      </c>
+      <c r="H210" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B211" t="str">
+        <v>12억 4,000</v>
+      </c>
+      <c r="C211">
+        <v>108</v>
+      </c>
+      <c r="D211" t="str">
+        <v>506동</v>
+      </c>
+      <c r="E211" t="str">
+        <v>22/25</v>
+      </c>
+      <c r="F211" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G211" t="str">
+        <v>프리미엄확장형, 빠른입주가능, 동천역세권</v>
+      </c>
+      <c r="H211" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B212" t="str">
+        <v>13억</v>
+      </c>
+      <c r="C212">
+        <v>108</v>
+      </c>
+      <c r="D212" t="str">
+        <v>514동</v>
+      </c>
+      <c r="E212" t="str">
+        <v>10/25</v>
+      </c>
+      <c r="F212" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G212" t="str">
+        <v>0318966776 최근확장올수리됨입주협의가능.</v>
+      </c>
+      <c r="H212" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B213" t="str">
+        <v>13억</v>
+      </c>
+      <c r="C213">
+        <v>108</v>
+      </c>
+      <c r="D213" t="str">
+        <v>512동</v>
+      </c>
+      <c r="E213" t="str">
+        <v>저/23</v>
+      </c>
+      <c r="F213" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G213" t="str">
+        <v>로얄동,로얄층,특올수리,특전망</v>
+      </c>
+      <c r="H213" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B214" t="str">
+        <v>12억 2,000</v>
+      </c>
+      <c r="C214">
+        <v>108</v>
+      </c>
+      <c r="D214" t="str">
+        <v>512동</v>
+      </c>
+      <c r="E214" t="str">
+        <v>중/23</v>
+      </c>
+      <c r="F214" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G214" t="str">
+        <v>로얄동 확장 깨끗  세안고</v>
+      </c>
+      <c r="H214" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B215" t="str">
+        <v>11억 7,000</v>
+      </c>
+      <c r="C215">
+        <v>108</v>
+      </c>
+      <c r="D215" t="str">
+        <v>510동</v>
+      </c>
+      <c r="E215" t="str">
+        <v>저/24</v>
+      </c>
+      <c r="F215" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G215" t="str">
+        <v>프리미엄확장.정상입주.동천역 도보 9분. 전자계약 가능</v>
+      </c>
+      <c r="H215" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B216" t="str">
+        <v>12억 3,000</v>
+      </c>
+      <c r="C216">
+        <v>108</v>
+      </c>
+      <c r="D216" t="str">
+        <v>515동</v>
+      </c>
+      <c r="E216" t="str">
+        <v>저/23</v>
+      </c>
+      <c r="F216" t="str">
+        <v>북서향</v>
+      </c>
+      <c r="G216" t="str">
+        <v>전체 확장 화이트올수리 입주가 탁트인정원전망 라인굿</v>
+      </c>
+      <c r="H216" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B217" t="str">
+        <v>12억 7,000</v>
+      </c>
+      <c r="C217">
+        <v>108</v>
+      </c>
+      <c r="D217" t="str">
+        <v>503동</v>
+      </c>
+      <c r="E217" t="str">
+        <v>25/25</v>
+      </c>
+      <c r="F217" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G217" t="str">
+        <v>o성실o프리미엄확장.전망굿탑층.실입주.로얄동.주인관리깨끗.동천역도보</v>
+      </c>
+      <c r="H217" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B218" t="str">
+        <v>12억</v>
+      </c>
+      <c r="C218">
+        <v>108</v>
+      </c>
+      <c r="D218" t="str">
+        <v>504동</v>
+      </c>
+      <c r="E218" t="str">
+        <v>2/25</v>
+      </c>
+      <c r="F218" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G218" t="str">
+        <v>0318966776 전망아주좋음확장수리잘됨</v>
+      </c>
+      <c r="H218" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B219" t="str">
+        <v>12억 2,000</v>
+      </c>
+      <c r="C219">
+        <v>108</v>
+      </c>
+      <c r="D219" t="str">
+        <v>515동</v>
+      </c>
+      <c r="E219" t="str">
+        <v>중/23</v>
+      </c>
+      <c r="F219" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G219" t="str">
+        <v>로얄동층 트인전망예뻐요 확장형 동천역과상가인접이라서 편해요</v>
+      </c>
+      <c r="H219" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B220" t="str">
+        <v>11억 1,000</v>
+      </c>
+      <c r="C220">
+        <v>108</v>
+      </c>
+      <c r="D220" t="str">
+        <v>501동</v>
+      </c>
+      <c r="E220" t="str">
+        <v>저/25</v>
+      </c>
+      <c r="F220" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G220" t="str">
+        <v>로얄동 출입동 입주협의가 깨끗 생활편리 동천역도보편리</v>
+      </c>
+      <c r="H220" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B221" t="str">
+        <v>12억 9,000</v>
+      </c>
+      <c r="C221">
+        <v>108</v>
+      </c>
+      <c r="D221" t="str">
+        <v>509동</v>
+      </c>
+      <c r="E221" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F221" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G221" t="str">
+        <v>특올수리 채광좋은고층 생활편리 로얄동 입주협의 소유주직접의뢰</v>
+      </c>
+      <c r="H221" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B222" t="str">
+        <v>12억 3,000</v>
+      </c>
+      <c r="C222">
+        <v>108</v>
+      </c>
+      <c r="D222" t="str">
+        <v>505동</v>
+      </c>
+      <c r="E222" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F222" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G222" t="str">
+        <v>확장형 채광좋은 관리잘된집 조율가 동천역도보10분</v>
+      </c>
+      <c r="H222" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B223" t="str">
+        <v>12억</v>
+      </c>
+      <c r="C223">
+        <v>108</v>
+      </c>
+      <c r="D223" t="str">
+        <v>504동</v>
+      </c>
+      <c r="E223" t="str">
+        <v>중/25</v>
+      </c>
+      <c r="F223" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G223" t="str">
+        <v>전망 좋은 로얄동,올확장,입주일 협의 가</v>
+      </c>
+      <c r="H223" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B224" t="str">
+        <v>12억 2,000</v>
+      </c>
+      <c r="C224">
+        <v>108</v>
+      </c>
+      <c r="D224" t="str">
+        <v>502동</v>
+      </c>
+      <c r="E224" t="str">
+        <v>중/21</v>
+      </c>
+      <c r="F224" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G224" t="str">
+        <v>올수리 프리미엄확장 로얄동층 트인불곡산전망 출입동생활편리</v>
+      </c>
+      <c r="H224" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B225" t="str">
+        <v>12억</v>
+      </c>
+      <c r="C225">
+        <v>108</v>
+      </c>
+      <c r="D225" t="str">
+        <v>509동</v>
+      </c>
+      <c r="E225" t="str">
+        <v>7/25</v>
+      </c>
+      <c r="F225" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G225" t="str">
+        <v>세안고, 파크뷰, 동천초, 산책로굿, 조용</v>
+      </c>
+      <c r="H225" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B226" t="str">
+        <v>12억 5,000</v>
+      </c>
+      <c r="C226">
+        <v>108</v>
+      </c>
+      <c r="D226" t="str">
+        <v>503동</v>
+      </c>
+      <c r="E226" t="str">
+        <v>중/25</v>
+      </c>
+      <c r="F226" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G226" t="str">
+        <v>로얄동층 트인불곡산전망 확장 화이트수리 관리최상 동천역도보편리</v>
+      </c>
+      <c r="H226" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B227" t="str">
+        <v>12억 3,000</v>
+      </c>
+      <c r="C227">
+        <v>108</v>
+      </c>
+      <c r="D227" t="str">
+        <v>515동</v>
+      </c>
+      <c r="E227" t="str">
+        <v>중/23</v>
+      </c>
+      <c r="F227" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G227" t="str">
+        <v>올확장  입주가능 탁트인뷰 채광굿</v>
+      </c>
+      <c r="H227" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B228" t="str">
+        <v>12억</v>
+      </c>
+      <c r="C228">
+        <v>108</v>
+      </c>
+      <c r="D228" t="str">
+        <v>505동</v>
+      </c>
+      <c r="E228" t="str">
+        <v>고/25</v>
+      </c>
+      <c r="F228" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G228" t="str">
+        <v>프리미엄확장,밝고 깔끔,학교까까운 동</v>
+      </c>
+      <c r="H228" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B229" t="str">
+        <v>13억</v>
+      </c>
+      <c r="C229">
+        <v>108</v>
+      </c>
+      <c r="D229" t="str">
+        <v>514동</v>
+      </c>
+      <c r="E229" t="str">
+        <v>중/25</v>
+      </c>
+      <c r="F229" t="str">
+        <v/>
+      </c>
+      <c r="G229" t="str">
+        <v>로얄동,트인뷰,프리미엄확장,깔끔관리</v>
+      </c>
+      <c r="H229" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B230" t="str">
+        <v>12억 4,000</v>
+      </c>
+      <c r="C230" t="str">
+        <v>108</v>
+      </c>
+      <c r="D230" t="str">
+        <v>506동</v>
+      </c>
+      <c r="E230" t="str">
+        <v>고층</v>
+      </c>
+      <c r="F230" t="str">
+        <v/>
+      </c>
+      <c r="G230" t="str">
+        <v>o성실o전체확장형.해잘들어밝아요.LED교체.깨끗해요.빠른입주가능</v>
+      </c>
+      <c r="H230" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B231" t="str">
+        <v>11억 2,000</v>
+      </c>
+      <c r="C231" t="str">
+        <v>108</v>
+      </c>
+      <c r="D231" t="str">
+        <v>506동</v>
+      </c>
+      <c r="E231" t="str">
+        <v>7층</v>
+      </c>
+      <c r="F231" t="str">
+        <v/>
+      </c>
+      <c r="G231" t="str">
+        <v>급매, 확장형, 공원전망 , 입주일자 협의가능</v>
+      </c>
+      <c r="H231" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B232" t="str">
+        <v>11억 5,000</v>
+      </c>
+      <c r="C232" t="str">
+        <v>108</v>
+      </c>
+      <c r="D232" t="str">
+        <v>511동</v>
+      </c>
+      <c r="E232" t="str">
+        <v>고층</v>
+      </c>
+      <c r="F232" t="str">
+        <v/>
+      </c>
+      <c r="G232" t="str">
+        <v>o.세안고27.3.27입주,탁트인전망,올확장,최근올수리,관리최상</v>
+      </c>
+      <c r="H232" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B233" t="str">
+        <v>12억 5,000</v>
+      </c>
+      <c r="C233" t="str">
+        <v>108</v>
+      </c>
+      <c r="D233" t="str">
+        <v>503동</v>
+      </c>
+      <c r="E233" t="str">
+        <v>25층</v>
+      </c>
+      <c r="F233" t="str">
+        <v/>
+      </c>
+      <c r="G233" t="str">
+        <v>탁트인로얄동 환상전망 프리미엄확장 상권교통편리한입구동 대단지</v>
+      </c>
+      <c r="H233" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>동천디이스트</v>
+      </c>
+      <c r="B234" t="str">
+        <v>12억 5,000</v>
+      </c>
+      <c r="C234" t="str">
+        <v>108</v>
+      </c>
+      <c r="D234" t="str">
+        <v>502동</v>
+      </c>
+      <c r="E234" t="str">
+        <v>중층</v>
+      </c>
+      <c r="F234" t="str">
+        <v/>
+      </c>
+      <c r="G234" t="str">
+        <v>로얄동층 완전트인뷰 프리미엄확장 입주협의가 출입동 동천역도보편리</v>
+      </c>
+      <c r="H234" t="str">
+        <v>asil</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B235" t="str">
+        <v>9억 3,000</v>
+      </c>
+      <c r="C235">
+        <v>92</v>
+      </c>
+      <c r="D235" t="str">
+        <v>106동</v>
+      </c>
+      <c r="E235" t="str">
+        <v>1/19</v>
+      </c>
+      <c r="F235" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G235" t="str">
+        <v>정상,깨끗하고 일부수리에 전망굿 단지내초등학교 신분당선 동천역10분</v>
+      </c>
+      <c r="H235" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B236" t="str">
+        <v>11억 2,000</v>
+      </c>
+      <c r="C236">
+        <v>109</v>
+      </c>
+      <c r="D236" t="str">
+        <v>107동</v>
+      </c>
+      <c r="E236" t="str">
+        <v>7/18</v>
+      </c>
+      <c r="F236" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G236" t="str">
+        <v>추천매물 로얄동 앞트인전망 결로 곰팡이없이 관리최상</v>
+      </c>
+      <c r="H236" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B237" t="str">
+        <v>10억</v>
+      </c>
+      <c r="C237">
+        <v>92</v>
+      </c>
+      <c r="D237" t="str">
+        <v>101동</v>
+      </c>
+      <c r="E237" t="str">
+        <v>13/15</v>
+      </c>
+      <c r="F237" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G237" t="str">
+        <v>28. 동천역 손곡초중 남향 방3화2 현재 세입자거주중 월세안고매매</v>
+      </c>
+      <c r="H237" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B238" t="str">
+        <v>10억 3,000</v>
+      </c>
+      <c r="C238">
+        <v>109</v>
+      </c>
+      <c r="D238" t="str">
+        <v>103동</v>
+      </c>
+      <c r="E238" t="str">
+        <v>1/19</v>
+      </c>
+      <c r="F238" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G238" t="str">
+        <v>초품아,방2확장 화이트수리,주인거주,강남판교 출퇴근 용이</v>
+      </c>
+      <c r="H238" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B239" t="str">
+        <v>11억</v>
+      </c>
+      <c r="C239">
+        <v>109</v>
+      </c>
+      <c r="D239" t="str">
+        <v>104동</v>
+      </c>
+      <c r="E239" t="str">
+        <v>7/19</v>
+      </c>
+      <c r="F239" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G239" t="str">
+        <v>로얄동 급매 짧은세안고</v>
+      </c>
+      <c r="H239" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B240" t="str">
+        <v>10억</v>
+      </c>
+      <c r="C240">
+        <v>92</v>
+      </c>
+      <c r="D240" t="str">
+        <v>106동</v>
+      </c>
+      <c r="E240" t="str">
+        <v>18/19</v>
+      </c>
+      <c r="F240" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G240" t="str">
+        <v>귀한매물 올확장 수리 전망트임</v>
+      </c>
+      <c r="H240" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B241" t="str">
+        <v>10억 3,000</v>
+      </c>
+      <c r="C241">
+        <v>109</v>
+      </c>
+      <c r="D241" t="str">
+        <v>105동</v>
+      </c>
+      <c r="E241" t="str">
+        <v>2/19</v>
+      </c>
+      <c r="F241" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G241" t="str">
+        <v>로얄동 5.1억 전세안고 매매 초품아 잔금일협의</v>
+      </c>
+      <c r="H241" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B242" t="str">
+        <v>10억</v>
+      </c>
+      <c r="C242">
+        <v>92</v>
+      </c>
+      <c r="D242" t="str">
+        <v>106동</v>
+      </c>
+      <c r="E242" t="str">
+        <v>고/19</v>
+      </c>
+      <c r="F242" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G242" t="str">
+        <v>정상,깨끗하고 전망굿 단지내초등학교 신분당선 동천역10분</v>
+      </c>
+      <c r="H242" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B243" t="str">
+        <v>11억 5,000</v>
+      </c>
+      <c r="C243">
+        <v>109</v>
+      </c>
+      <c r="D243" t="str">
+        <v>107동</v>
+      </c>
+      <c r="E243" t="str">
+        <v>17/18</v>
+      </c>
+      <c r="F243" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G243" t="str">
+        <v>로얄동 전망최고 수리됨</v>
+      </c>
+      <c r="H243" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B244" t="str">
+        <v>10억</v>
+      </c>
+      <c r="C244">
+        <v>109</v>
+      </c>
+      <c r="D244" t="str">
+        <v>105동</v>
+      </c>
+      <c r="E244" t="str">
+        <v>1/19</v>
+      </c>
+      <c r="F244" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G244" t="str">
+        <v>따스한남향 방확장 주인거주 채광굿 깔끔관리</v>
+      </c>
+      <c r="H244" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>써니벨리</v>
+      </c>
+      <c r="B245" t="str">
+        <v>10억 2,000</v>
+      </c>
+      <c r="C245">
+        <v>109</v>
+      </c>
+      <c r="D245" t="str">
+        <v>102동</v>
+      </c>
+      <c r="E245" t="str">
+        <v>3/14</v>
+      </c>
+      <c r="F245" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G245" t="str">
+        <v>남향 확장 세안고</v>
+      </c>
+      <c r="H245" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B246" t="str">
+        <v>13억</v>
+      </c>
+      <c r="C246">
+        <v>163</v>
+      </c>
+      <c r="D246" t="str">
+        <v>107동</v>
+      </c>
+      <c r="E246" t="str">
+        <v>15/18</v>
+      </c>
+      <c r="F246" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G246" t="str">
+        <v>강추,49형,로얄동,화이트올수리,깨끗한집.초역세권,세안고다주택자</v>
+      </c>
+      <c r="H246" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B247" t="str">
+        <v>14억 5,000</v>
+      </c>
+      <c r="C247">
+        <v>163</v>
+      </c>
+      <c r="D247" t="str">
+        <v>107동</v>
+      </c>
+      <c r="E247" t="str">
+        <v>6/18</v>
+      </c>
+      <c r="F247" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G247" t="str">
+        <v>로얄동 트인전망  초역세권 생활권좋음 세안고</v>
+      </c>
+      <c r="H247" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B248" t="str">
+        <v>14억 3,000</v>
+      </c>
+      <c r="C248">
+        <v>195</v>
+      </c>
+      <c r="D248" t="str">
+        <v>101동</v>
+      </c>
+      <c r="E248" t="str">
+        <v>18/18</v>
+      </c>
+      <c r="F248" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G248" t="str">
+        <v>입구동 전망굿 초역세권 화장실2수리</v>
+      </c>
+      <c r="H248" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B249" t="str">
+        <v>14억 5,000</v>
+      </c>
+      <c r="C249">
+        <v>163</v>
+      </c>
+      <c r="D249" t="str">
+        <v>105동</v>
+      </c>
+      <c r="E249" t="str">
+        <v>중/18</v>
+      </c>
+      <c r="F249" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G249" t="str">
+        <v>샷시포함특올수리 성복역세권 생활편리 학군최고</v>
+      </c>
+      <c r="H249" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B250" t="str">
+        <v>12억</v>
+      </c>
+      <c r="C250">
+        <v>109</v>
+      </c>
+      <c r="D250" t="str">
+        <v>103동</v>
+      </c>
+      <c r="E250" t="str">
+        <v>중/18</v>
+      </c>
+      <c r="F250" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G250" t="str">
+        <v>정상입주,방확장,주방씽크대외수리함.성복역초역세권</v>
+      </c>
+      <c r="H250" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B251" t="str">
+        <v>11억 5,000</v>
+      </c>
+      <c r="C251">
+        <v>109</v>
+      </c>
+      <c r="D251" t="str">
+        <v>103동</v>
+      </c>
+      <c r="E251" t="str">
+        <v>11/18</v>
+      </c>
+      <c r="F251" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G251" t="str">
+        <v>올수리 폴딩도어 정상입주 성복역 도보2분 생활권좋음</v>
+      </c>
+      <c r="H251" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B252" t="str">
+        <v>13억 5,000</v>
+      </c>
+      <c r="C252">
+        <v>163</v>
+      </c>
+      <c r="D252" t="str">
+        <v>105동</v>
+      </c>
+      <c r="E252" t="str">
+        <v>7/18</v>
+      </c>
+      <c r="F252" t="str">
+        <v>남향</v>
+      </c>
+      <c r="G252" t="str">
+        <v>세안고 남향 성복역 도보2분 상권인접 기본</v>
+      </c>
+      <c r="H252" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B253" t="str">
+        <v>13억 5,000</v>
+      </c>
+      <c r="C253">
+        <v>163</v>
+      </c>
+      <c r="D253" t="str">
+        <v>106동</v>
+      </c>
+      <c r="E253" t="str">
+        <v>12/18</v>
+      </c>
+      <c r="F253" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G253" t="str">
+        <v>채광굿 초역세권 도보2분 생활권 좋음  기본</v>
+      </c>
+      <c r="H253" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B254" t="str">
+        <v>11억 2,000</v>
+      </c>
+      <c r="C254">
+        <v>109</v>
+      </c>
+      <c r="D254" t="str">
+        <v>104동</v>
+      </c>
+      <c r="E254" t="str">
+        <v>10/18</v>
+      </c>
+      <c r="F254" t="str">
+        <v>남동향</v>
+      </c>
+      <c r="G254" t="str">
+        <v>거실확장 방1확장 올수리 초역세권 도보3분 상권인접</v>
+      </c>
+      <c r="H254" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B255" t="str">
+        <v>15억</v>
+      </c>
+      <c r="C255">
+        <v>195</v>
+      </c>
+      <c r="D255" t="str">
+        <v>101동</v>
+      </c>
+      <c r="E255" t="str">
+        <v>고/18</v>
+      </c>
+      <c r="F255" t="str">
+        <v>남서향</v>
+      </c>
+      <c r="G255" t="str">
+        <v>깨끗하고 해잘드는 이쁜집</v>
+      </c>
+      <c r="H255" t="str">
+        <v>naver</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>성동마을강남</v>
+      </c>
+      <c r="B256" t="str">
+        <v>12억 9,000</v>
+      </c>
+      <c r="C256" t="str">
+        <v>163</v>
+      </c>
+      <c r="D256" t="str">
+        <v>107동</v>
+      </c>
+      <c r="E256" t="str">
+        <v>15층</v>
+      </c>
+      <c r="F256" t="str">
+        <v/>
+      </c>
+      <c r="G256" t="str">
+        <v>무주택자, 세안고, 남향, 화이트 올수리, 트인 조망, 성복역 도보5분</v>
+      </c>
+      <c r="H256" t="str">
+        <v>asil</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H172"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H256"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>